<commit_message>
add dcase 2023 paper
</commit_message>
<xml_diff>
--- a/markdown_generator/publications.xlsx
+++ b/markdown_generator/publications.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mcartwright/git/sinc-laboratory.github.io/markdown_generator/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sripathisridhar/Documents/code/sinc-laboratory.github.io/markdown_generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FAEE6D0-6406-8B44-96BA-A0CF51757F56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC652C4E-87EE-F54A-A6CB-481A1EA3DB89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2100" yWindow="2480" windowWidth="27740" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2100" yWindow="2140" windowWidth="27740" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="publications" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="348">
   <si>
     <t>title</t>
   </si>
@@ -1049,6 +1049,21 @@
   </si>
   <si>
     <t>right</t>
+  </si>
+  <si>
+    <t>Multi-label Open-set Audio Classification</t>
+  </si>
+  <si>
+    <t>sridhar2023multi.pdf</t>
+  </si>
+  <si>
+    <t>Current audio classification models have small class vocabularies relative to the large number of sound event classes of interest in the real world. Thus, they provide a limited view of the world that may miss important yet unexpected or unknown sound events. To address this issue, open-set audio classification techniques have been developed to detect sound events from unknown classes. Although these methods have been applied to a multi-class context in audio, such as sound scene classification, they have yet to be investigated for polyphonic audio in which sound events overlap, requiring the use of multi-label models. In this study, we establish the problem of multi-label open-set audio classification by creating a dataset with varying unknown class distributions and evaluating baseline approaches built upon existing techniques.</t>
+  </si>
+  <si>
+    <t>sridhar_dcase23_model.png</t>
+  </si>
+  <si>
+    <t>Sridhar, S., and Cartwright, M. Multi-label Open-set Audio Classification. In &lt;i&gt;Proceedings of the Workshop on Detection and Classification of Acoustic Scenes and Events (DCASE)&lt;/i&gt;, 2023.</t>
   </si>
 </sst>
 </file>
@@ -1551,13 +1566,11 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1618,9 +1631,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1658,7 +1671,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1764,7 +1777,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1906,7 +1919,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1914,18 +1927,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R46"/>
+  <dimension ref="A1:R47"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="3"/>
+    <col min="1" max="1" width="10.83203125" style="2"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
     <col min="3" max="4" width="76.6640625" customWidth="1"/>
     <col min="6" max="6" width="51.1640625" customWidth="1"/>
-    <col min="7" max="7" width="73.33203125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="73.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>167</v>
       </c>
       <c r="B1" t="s">
@@ -1943,7 +1956,7 @@
       <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" t="s">
         <v>4</v>
       </c>
       <c r="H1" t="s">
@@ -1981,7 +1994,7 @@
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A2" s="3">
+      <c r="A2" s="2">
         <v>43678</v>
       </c>
       <c r="B2" t="s">
@@ -1999,7 +2012,7 @@
       <c r="F2" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" t="s">
         <v>9</v>
       </c>
       <c r="R2" t="s">
@@ -2007,7 +2020,7 @@
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A3" s="3">
+      <c r="A3" s="2">
         <v>43739</v>
       </c>
       <c r="B3" t="s">
@@ -2025,7 +2038,7 @@
       <c r="F3" t="s">
         <v>12</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" t="s">
         <v>13</v>
       </c>
       <c r="H3" t="s">
@@ -2048,7 +2061,7 @@
       </c>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A4" s="3">
+      <c r="A4" s="2">
         <v>43739</v>
       </c>
       <c r="B4" t="s">
@@ -2066,7 +2079,7 @@
       <c r="F4" t="s">
         <v>19</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" t="s">
         <v>20</v>
       </c>
       <c r="H4" t="s">
@@ -2086,7 +2099,7 @@
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A5" s="3">
+      <c r="A5" s="2">
         <v>43739</v>
       </c>
       <c r="B5" t="s">
@@ -2104,7 +2117,7 @@
       <c r="F5" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="G5" t="s">
         <v>200</v>
       </c>
       <c r="H5" t="s">
@@ -2121,7 +2134,7 @@
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A6" s="3">
+      <c r="A6" s="2">
         <v>43466</v>
       </c>
       <c r="B6" t="s">
@@ -2139,13 +2152,13 @@
       <c r="F6" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" t="s">
         <v>30</v>
       </c>
       <c r="H6" t="s">
         <v>31</v>
       </c>
-      <c r="J6" s="5">
+      <c r="J6">
         <v>66</v>
       </c>
       <c r="N6" t="s">
@@ -2159,7 +2172,7 @@
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A7" s="3">
+      <c r="A7" s="2">
         <v>43586</v>
       </c>
       <c r="B7" t="s">
@@ -2177,7 +2190,7 @@
       <c r="F7" t="s">
         <v>34</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G7" t="s">
         <v>35</v>
       </c>
       <c r="R7" t="s">
@@ -2185,7 +2198,7 @@
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A8" s="3">
+      <c r="A8" s="2">
         <v>43556</v>
       </c>
       <c r="B8" t="s">
@@ -2203,7 +2216,7 @@
       <c r="F8" t="s">
         <v>38</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" t="s">
         <v>39</v>
       </c>
       <c r="H8" t="s">
@@ -2220,7 +2233,7 @@
       </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A9" s="3">
+      <c r="A9" s="2">
         <v>43556</v>
       </c>
       <c r="B9" t="s">
@@ -2238,7 +2251,7 @@
       <c r="F9" t="s">
         <v>42</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G9" t="s">
         <v>43</v>
       </c>
       <c r="H9" t="s">
@@ -2255,7 +2268,7 @@
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A10" s="3">
+      <c r="A10" s="2">
         <v>43466</v>
       </c>
       <c r="B10" t="s">
@@ -2273,7 +2286,7 @@
       <c r="F10" t="s">
         <v>49</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" t="s">
         <v>50</v>
       </c>
       <c r="R10" t="s">
@@ -2281,7 +2294,7 @@
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A11" s="3">
+      <c r="A11" s="2">
         <v>43466</v>
       </c>
       <c r="B11" t="s">
@@ -2299,7 +2312,7 @@
       <c r="F11" t="s">
         <v>54</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="G11" t="s">
         <v>55</v>
       </c>
       <c r="R11" t="s">
@@ -2307,7 +2320,7 @@
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A12" s="3">
+      <c r="A12" s="2">
         <v>43344</v>
       </c>
       <c r="B12" t="s">
@@ -2325,7 +2338,7 @@
       <c r="F12" t="s">
         <v>58</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" t="s">
         <v>59</v>
       </c>
       <c r="H12" t="s">
@@ -2348,7 +2361,7 @@
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A13" s="3">
+      <c r="A13" s="2">
         <v>43191</v>
       </c>
       <c r="B13" t="s">
@@ -2366,7 +2379,7 @@
       <c r="F13" t="s">
         <v>65</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="G13" t="s">
         <v>130</v>
       </c>
       <c r="H13" t="s">
@@ -2392,7 +2405,7 @@
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A14" s="3">
+      <c r="A14" s="2">
         <v>43191</v>
       </c>
       <c r="B14" t="s">
@@ -2410,7 +2423,7 @@
       <c r="F14" t="s">
         <v>68</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="G14" t="s">
         <v>133</v>
       </c>
       <c r="L14" t="s">
@@ -2424,7 +2437,7 @@
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A15" s="3">
+      <c r="A15" s="2">
         <v>43040</v>
       </c>
       <c r="B15" t="s">
@@ -2442,7 +2455,7 @@
       <c r="F15" t="s">
         <v>72</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="G15" t="s">
         <v>139</v>
       </c>
       <c r="H15" t="s">
@@ -2471,7 +2484,7 @@
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A16" s="3">
+      <c r="A16" s="2">
         <v>43009</v>
       </c>
       <c r="B16" t="s">
@@ -2489,13 +2502,13 @@
       <c r="F16" t="s">
         <v>75</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="G16" t="s">
         <v>141</v>
       </c>
       <c r="H16" t="s">
         <v>142</v>
       </c>
-      <c r="J16" s="5">
+      <c r="J16">
         <v>50</v>
       </c>
       <c r="N16" s="1" t="s">
@@ -2515,7 +2528,7 @@
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A17" s="3">
+      <c r="A17" s="2">
         <v>42705</v>
       </c>
       <c r="B17" t="s">
@@ -2533,7 +2546,7 @@
       <c r="F17" t="s">
         <v>79</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="G17" t="s">
         <v>173</v>
       </c>
       <c r="R17" t="s">
@@ -2541,7 +2554,7 @@
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A18" s="3">
+      <c r="A18" s="2">
         <v>42583</v>
       </c>
       <c r="B18" t="s">
@@ -2559,7 +2572,7 @@
       <c r="F18" t="s">
         <v>82</v>
       </c>
-      <c r="G18" s="2" t="s">
+      <c r="G18" t="s">
         <v>145</v>
       </c>
       <c r="R18" t="s">
@@ -2567,7 +2580,7 @@
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A19" s="3">
+      <c r="A19" s="2">
         <v>42491</v>
       </c>
       <c r="B19" t="s">
@@ -2585,7 +2598,7 @@
       <c r="F19" t="s">
         <v>85</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="G19" t="s">
         <v>146</v>
       </c>
       <c r="R19" t="s">
@@ -2593,7 +2606,7 @@
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A20" s="3">
+      <c r="A20" s="2">
         <v>42461</v>
       </c>
       <c r="B20" t="s">
@@ -2611,7 +2624,7 @@
       <c r="F20" t="s">
         <v>88</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="G20" t="s">
         <v>147</v>
       </c>
       <c r="H20" t="s">
@@ -2637,7 +2650,7 @@
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A21" s="3">
+      <c r="A21" s="2">
         <v>42278</v>
       </c>
       <c r="B21" t="s">
@@ -2655,13 +2668,13 @@
       <c r="F21" t="s">
         <v>91</v>
       </c>
-      <c r="G21" s="2" t="s">
+      <c r="G21" t="s">
         <v>149</v>
       </c>
-      <c r="H21" s="2" t="s">
+      <c r="H21" t="s">
         <v>188</v>
       </c>
-      <c r="I21" s="2" t="s">
+      <c r="I21" t="s">
         <v>185</v>
       </c>
       <c r="J21">
@@ -2672,7 +2685,7 @@
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A22" s="3">
+      <c r="A22" s="2">
         <v>42125</v>
       </c>
       <c r="B22" t="s">
@@ -2690,7 +2703,7 @@
       <c r="F22" t="s">
         <v>93</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="G22" t="s">
         <v>150</v>
       </c>
       <c r="H22" t="s">
@@ -2713,7 +2726,7 @@
       </c>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A23" s="3">
+      <c r="A23" s="2">
         <v>42125</v>
       </c>
       <c r="B23" t="s">
@@ -2731,7 +2744,7 @@
       <c r="F23" t="s">
         <v>96</v>
       </c>
-      <c r="G23" s="2" t="s">
+      <c r="G23" t="s">
         <v>153</v>
       </c>
       <c r="R23" t="s">
@@ -2739,7 +2752,7 @@
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A24" s="3">
+      <c r="A24" s="2">
         <v>41944</v>
       </c>
       <c r="B24" t="s">
@@ -2757,7 +2770,7 @@
       <c r="F24" t="s">
         <v>98</v>
       </c>
-      <c r="G24" s="2" t="s">
+      <c r="G24" t="s">
         <v>156</v>
       </c>
       <c r="K24" t="s">
@@ -2768,7 +2781,7 @@
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A25" s="3">
+      <c r="A25" s="2">
         <v>41821</v>
       </c>
       <c r="B25" t="s">
@@ -2786,7 +2799,7 @@
       <c r="F25" t="s">
         <v>100</v>
       </c>
-      <c r="G25" s="2" t="s">
+      <c r="G25" t="s">
         <v>157</v>
       </c>
       <c r="K25" t="s">
@@ -2797,7 +2810,7 @@
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A26" s="3">
+      <c r="A26" s="2">
         <v>41760</v>
       </c>
       <c r="B26" t="s">
@@ -2815,7 +2828,7 @@
       <c r="F26" t="s">
         <v>104</v>
       </c>
-      <c r="G26" s="2" t="s">
+      <c r="G26" t="s">
         <v>174</v>
       </c>
       <c r="R26" t="s">
@@ -2823,7 +2836,7 @@
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A27" s="3">
+      <c r="A27" s="2">
         <v>41730</v>
       </c>
       <c r="B27" t="s">
@@ -2841,7 +2854,7 @@
       <c r="F27" t="s">
         <v>107</v>
       </c>
-      <c r="G27" s="2" t="s">
+      <c r="G27" t="s">
         <v>158</v>
       </c>
       <c r="K27" t="s">
@@ -2852,7 +2865,7 @@
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A28" s="3">
+      <c r="A28" s="2">
         <v>41579</v>
       </c>
       <c r="B28" t="s">
@@ -2870,7 +2883,7 @@
       <c r="F28" t="s">
         <v>110</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="G28" t="s">
         <v>159</v>
       </c>
       <c r="H28" t="s">
@@ -2884,7 +2897,7 @@
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A29" s="3">
+      <c r="A29" s="2">
         <v>41214</v>
       </c>
       <c r="B29" t="s">
@@ -2902,7 +2915,7 @@
       <c r="F29" t="s">
         <v>113</v>
       </c>
-      <c r="G29" s="2" t="s">
+      <c r="G29" t="s">
         <v>160</v>
       </c>
       <c r="R29" t="s">
@@ -2910,7 +2923,7 @@
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A30" s="3">
+      <c r="A30" s="2">
         <v>41091</v>
       </c>
       <c r="B30" t="s">
@@ -2928,7 +2941,7 @@
       <c r="F30" t="s">
         <v>116</v>
       </c>
-      <c r="G30" s="2" t="s">
+      <c r="G30" t="s">
         <v>161</v>
       </c>
       <c r="R30" t="s">
@@ -2936,7 +2949,7 @@
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A31" s="3">
+      <c r="A31" s="2">
         <v>40848</v>
       </c>
       <c r="B31" t="s">
@@ -2954,7 +2967,7 @@
       <c r="F31" t="s">
         <v>120</v>
       </c>
-      <c r="G31" s="2" t="s">
+      <c r="G31" t="s">
         <v>162</v>
       </c>
       <c r="R31" t="s">
@@ -2962,7 +2975,7 @@
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A32" s="3">
+      <c r="A32" s="2">
         <v>40634</v>
       </c>
       <c r="B32" t="s">
@@ -2980,7 +2993,7 @@
       <c r="F32" t="s">
         <v>123</v>
       </c>
-      <c r="G32" s="2" t="s">
+      <c r="G32" t="s">
         <v>163</v>
       </c>
       <c r="R32" t="s">
@@ -2988,7 +3001,7 @@
       </c>
     </row>
     <row r="33" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A33" s="3">
+      <c r="A33" s="2">
         <v>40360</v>
       </c>
       <c r="B33" t="s">
@@ -3006,7 +3019,7 @@
       <c r="F33" t="s">
         <v>126</v>
       </c>
-      <c r="G33" s="2" t="s">
+      <c r="G33" t="s">
         <v>164</v>
       </c>
       <c r="H33" t="s">
@@ -3029,7 +3042,7 @@
       </c>
     </row>
     <row r="34" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A34" s="3">
+      <c r="A34" s="2">
         <v>39264</v>
       </c>
       <c r="B34" t="s">
@@ -3047,7 +3060,7 @@
       <c r="F34" t="s">
         <v>129</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="G34" t="s">
         <v>165</v>
       </c>
       <c r="R34" t="s">
@@ -3055,7 +3068,7 @@
       </c>
     </row>
     <row r="35" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A35" s="3">
+      <c r="A35" s="2">
         <v>44137</v>
       </c>
       <c r="B35" t="s">
@@ -3073,7 +3086,7 @@
       <c r="F35" t="s">
         <v>204</v>
       </c>
-      <c r="G35" s="2" t="s">
+      <c r="G35" t="s">
         <v>201</v>
       </c>
       <c r="H35" t="s">
@@ -3102,7 +3115,7 @@
       </c>
     </row>
     <row r="36" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A36" s="3">
+      <c r="A36" s="2">
         <v>44115</v>
       </c>
       <c r="B36" t="s">
@@ -3120,10 +3133,10 @@
       <c r="F36" t="s">
         <v>215</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="G36" t="s">
         <v>213</v>
       </c>
-      <c r="H36" s="2" t="s">
+      <c r="H36" t="s">
         <v>214</v>
       </c>
       <c r="J36">
@@ -3140,7 +3153,7 @@
       </c>
     </row>
     <row r="37" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A37" s="3">
+      <c r="A37" s="2">
         <v>44355</v>
       </c>
       <c r="B37" t="s">
@@ -3158,10 +3171,10 @@
       <c r="F37" t="s">
         <v>217</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="G37" t="s">
         <v>216</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="H37" t="s">
         <v>220</v>
       </c>
       <c r="J37">
@@ -3175,7 +3188,7 @@
       </c>
     </row>
     <row r="38" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A38" s="3">
+      <c r="A38" s="2">
         <v>44355</v>
       </c>
       <c r="B38" t="s">
@@ -3193,10 +3206,10 @@
       <c r="F38" t="s">
         <v>224</v>
       </c>
-      <c r="G38" s="2" t="s">
+      <c r="G38" t="s">
         <v>228</v>
       </c>
-      <c r="H38" s="2" t="s">
+      <c r="H38" t="s">
         <v>225</v>
       </c>
       <c r="J38">
@@ -3219,16 +3232,16 @@
       </c>
     </row>
     <row r="39" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A39" s="3">
+      <c r="A39" s="2">
         <v>44486</v>
       </c>
       <c r="B39" t="s">
         <v>279</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C39" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="D39" s="4" t="s">
+      <c r="D39" s="3" t="s">
         <v>295</v>
       </c>
       <c r="E39" t="s">
@@ -3237,7 +3250,7 @@
       <c r="F39" t="s">
         <v>232</v>
       </c>
-      <c r="G39" s="2" t="s">
+      <c r="G39" t="s">
         <v>248</v>
       </c>
       <c r="H39" t="s">
@@ -3266,16 +3279,16 @@
       </c>
     </row>
     <row r="40" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A40" s="3">
+      <c r="A40" s="2">
         <v>44486</v>
       </c>
       <c r="B40" t="s">
         <v>240</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="D40" s="4" t="s">
+      <c r="D40" s="3" t="s">
         <v>295</v>
       </c>
       <c r="E40" t="s">
@@ -3284,7 +3297,7 @@
       <c r="F40" t="s">
         <v>242</v>
       </c>
-      <c r="G40" s="2" t="s">
+      <c r="G40" t="s">
         <v>239</v>
       </c>
       <c r="H40" t="s">
@@ -3313,7 +3326,7 @@
       </c>
     </row>
     <row r="41" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A41" s="3">
+      <c r="A41" s="2">
         <v>44493</v>
       </c>
       <c r="B41" t="s">
@@ -3331,7 +3344,7 @@
       <c r="F41" t="s">
         <v>255</v>
       </c>
-      <c r="G41" s="2" t="s">
+      <c r="G41" t="s">
         <v>256</v>
       </c>
       <c r="L41" t="s">
@@ -3351,7 +3364,7 @@
       </c>
     </row>
     <row r="42" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A42" s="3">
+      <c r="A42" s="2">
         <v>44802</v>
       </c>
       <c r="B42" t="s">
@@ -3369,10 +3382,10 @@
       <c r="F42" t="s">
         <v>264</v>
       </c>
-      <c r="G42" s="2" t="s">
+      <c r="G42" t="s">
         <v>263</v>
       </c>
-      <c r="H42" s="2" t="s">
+      <c r="H42" t="s">
         <v>265</v>
       </c>
       <c r="J42">
@@ -3386,7 +3399,7 @@
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A43" s="3">
+      <c r="A43" s="2">
         <v>44652</v>
       </c>
       <c r="B43" t="s">
@@ -3404,7 +3417,7 @@
       <c r="F43" t="s">
         <v>269</v>
       </c>
-      <c r="G43" s="2" t="s">
+      <c r="G43" t="s">
         <v>270</v>
       </c>
       <c r="H43" t="s">
@@ -3418,7 +3431,7 @@
       </c>
     </row>
     <row r="44" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A44" s="3">
+      <c r="A44" s="2">
         <v>44822</v>
       </c>
       <c r="B44" t="s">
@@ -3436,7 +3449,7 @@
       <c r="F44" t="s">
         <v>276</v>
       </c>
-      <c r="G44" s="2" t="s">
+      <c r="G44" t="s">
         <v>272</v>
       </c>
       <c r="R44" t="s">
@@ -3444,7 +3457,7 @@
       </c>
     </row>
     <row r="45" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A45" s="3">
+      <c r="A45" s="2">
         <v>44725</v>
       </c>
       <c r="B45" t="s">
@@ -3462,10 +3475,10 @@
       <c r="F45" t="s">
         <v>280</v>
       </c>
-      <c r="G45" s="2" t="s">
+      <c r="G45" t="s">
         <v>277</v>
       </c>
-      <c r="H45" s="2" t="s">
+      <c r="H45" t="s">
         <v>281</v>
       </c>
       <c r="J45">
@@ -3476,7 +3489,7 @@
       </c>
     </row>
     <row r="46" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A46" s="3">
+      <c r="A46" s="2">
         <v>44851</v>
       </c>
       <c r="B46" t="s">
@@ -3494,11 +3507,43 @@
       <c r="F46" t="s">
         <v>286</v>
       </c>
-      <c r="G46" s="2" t="s">
+      <c r="G46" t="s">
         <v>283</v>
       </c>
       <c r="R46" t="s">
         <v>292</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A47" s="2">
+        <v>45190</v>
+      </c>
+      <c r="B47" t="s">
+        <v>343</v>
+      </c>
+      <c r="C47" t="s">
+        <v>320</v>
+      </c>
+      <c r="D47" t="s">
+        <v>294</v>
+      </c>
+      <c r="E47" t="s">
+        <v>347</v>
+      </c>
+      <c r="F47" t="s">
+        <v>344</v>
+      </c>
+      <c r="G47" t="s">
+        <v>345</v>
+      </c>
+      <c r="H47" t="s">
+        <v>346</v>
+      </c>
+      <c r="J47">
+        <v>75</v>
+      </c>
+      <c r="R47" t="s">
+        <v>289</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add icassp 2025 paper
</commit_message>
<xml_diff>
--- a/markdown_generator/publications.xlsx
+++ b/markdown_generator/publications.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10413"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sripathisridhar/Documents/code/sinc-laboratory.github.io/markdown_generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC652C4E-87EE-F54A-A6CB-481A1EA3DB89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A0AAE53-DFA3-5E4A-877E-BBFD5CAE991D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2100" yWindow="2140" windowWidth="27740" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32680" yWindow="-2820" windowWidth="27740" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="publications" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="433" uniqueCount="348">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="356">
   <si>
     <t>title</t>
   </si>
@@ -1064,6 +1064,30 @@
   </si>
   <si>
     <t>Sridhar, S., and Cartwright, M. Multi-label Open-set Audio Classification. In &lt;i&gt;Proceedings of the Workshop on Detection and Classification of Acoustic Scenes and Events (DCASE)&lt;/i&gt;, 2023.</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.5281/zenodo.13755902</t>
+  </si>
+  <si>
+    <t>Open-set Tagging (OST) dataset</t>
+  </si>
+  <si>
+    <t>sridhar_icassp25_overview.png</t>
+  </si>
+  <si>
+    <t>sridhar2025compositional_poster.pdf</t>
+  </si>
+  <si>
+    <t>Human auditory perception is compositional in nature — we identify auditory streams from auditory scenes with multiple sound events. However, such auditory scenes are typically represented using clip-level representations that do not disentangle the constituent sound sources. In this work, we learn source-centric audio representations where each sound source is represented using a distinct, disentangled source embedding in the audio representation. We propose two novel approaches to learning source-centric audio representations: a supervised model guided by classification and an unsupervised model guided by feature reconstruction, both of which outperform the baselines. We thoroughly evaluate the design choices of both approaches using an audio classification task. We find that supervision is beneficial to learn source-centric representations, and that reconstructing audio features is more useful than reconstructing spectrograms to learn unsupervised source-centric representations. Leveraging source-centric models can help unlock the potential of greater interpretability and more flexible decoding in machine listening.</t>
+  </si>
+  <si>
+    <t>sridhar2025compositional.pdf</t>
+  </si>
+  <si>
+    <t>Compositional Audio Representation Learning</t>
+  </si>
+  <si>
+    <t>Sridhar, S., &amp; Cartwright, M. (2025, April). Compositional Audio Representation Learning. In ICASSP 2025-2025 IEEE International Conference on Acoustics, Speech and Signal Processing (ICASSP) (pp. 1-5). IEEE.</t>
   </si>
 </sst>
 </file>
@@ -1566,11 +1590,14 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1927,7 +1954,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R47"/>
+  <dimension ref="A1:R48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="2"/>
@@ -3543,6 +3570,47 @@
         <v>75</v>
       </c>
       <c r="R47" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="2">
+        <v>45753</v>
+      </c>
+      <c r="B48" t="s">
+        <v>354</v>
+      </c>
+      <c r="C48" t="s">
+        <v>324</v>
+      </c>
+      <c r="D48" t="s">
+        <v>298</v>
+      </c>
+      <c r="E48" t="s">
+        <v>355</v>
+      </c>
+      <c r="F48" t="s">
+        <v>353</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="H48" t="s">
+        <v>350</v>
+      </c>
+      <c r="J48">
+        <v>75</v>
+      </c>
+      <c r="L48" t="s">
+        <v>351</v>
+      </c>
+      <c r="P48" t="s">
+        <v>348</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>349</v>
+      </c>
+      <c r="R48" t="s">
         <v>289</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix icassp paper cite
</commit_message>
<xml_diff>
--- a/markdown_generator/publications.xlsx
+++ b/markdown_generator/publications.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sripathisridhar/Documents/code/sinc-laboratory.github.io/markdown_generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A0AAE53-DFA3-5E4A-877E-BBFD5CAE991D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A57057-2527-B64A-8885-A7C5186D7556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32680" yWindow="-2820" windowWidth="27740" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="publications" sheetId="1" r:id="rId1"/>
@@ -1087,7 +1087,7 @@
     <t>Compositional Audio Representation Learning</t>
   </si>
   <si>
-    <t>Sridhar, S., &amp; Cartwright, M. (2025, April). Compositional Audio Representation Learning. In ICASSP 2025-2025 IEEE International Conference on Acoustics, Speech and Signal Processing (ICASSP) (pp. 1-5). IEEE.</t>
+    <t>Sridhar, S., and Cartwright, M. Compositional Audio Representation Learning. In &lt;i&gt;Proceedings of the IEEE International Conference on Acoustics, Speech and Signal Processing (ICASSP)&lt;/i&gt;, 2025.</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Add Keita's publications CHI2024 and 2025
</commit_message>
<xml_diff>
--- a/markdown_generator/publications.xlsx
+++ b/markdown_generator/publications.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10611"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sripathisridhar/Documents/code/sinc-laboratory.github.io/markdown_generator/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/keitaohshiro/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8A57057-2527-B64A-8885-A7C5186D7556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B95927-D7FB-414D-BF49-D44C64D3CEAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="publications" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="444" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="365">
   <si>
     <t>title</t>
   </si>
@@ -1088,6 +1088,33 @@
   </si>
   <si>
     <t>Sridhar, S., and Cartwright, M. Compositional Audio Representation Learning. In &lt;i&gt;Proceedings of the IEEE International Conference on Acoustics, Speech and Signal Processing (ICASSP)&lt;/i&gt;, 2025.</t>
+  </si>
+  <si>
+    <t>Audio engineering by people who are deaf and hard of hearing: balancing confidence and limitations</t>
+  </si>
+  <si>
+    <t>ohshiro2024audioengineering.pdf</t>
+  </si>
+  <si>
+    <t>With technological advancements, audio engineering has evolved from a domain exclusive to professionals to one open to amateurs. However, research is limited on the accessibility of audio engineering, particularly for deaf, Deaf, and hard of hearing (DHH) individuals. To bridge this gap, we interviewed eight deaf and hard of hearing (dHH) audio engineers in music to understand accessibility in audio engineering. We found that their hearing magnified challenges in audio engineering: insecurities in sound perception undermined their confidence, and the required extra “hearing work” added complexity. As workarounds, participants employed various technologies and techniques, relied on the support of hearing peers, and developed strategies for learning and growth. Through these practices, they navigate audio engineering while balancing confidence and limitations. For future directions, we recommend exploring technologies that reduce insecurities and “hearing work” to empower DHH audio engineers and working toward a DHH-community-driven approach to accessible audio engineering.</t>
+  </si>
+  <si>
+    <t>ohshiro2025audioengineering_poster.pdf</t>
+  </si>
+  <si>
+    <t>Audio Engineering for Podcasts by deaf and Hard of Hearing Creators</t>
+  </si>
+  <si>
+    <t>Ohshiro, K., Cartwright, M. Audio Engineering for Podcasts by deaf and Hard of Hearing Creators. In &lt;i&gt;Proceedings of the ACM Conference on Human Factors in Computing Systems (CHI)&lt;/i&gt;, 2025.</t>
+  </si>
+  <si>
+    <t>Ohshiro, K., Cartwright, M. Audio engineering by people who are deaf and hard of hearing: balancing confidence and limitations. In &lt;i&gt;Proceedings of the ACM Conference on Human Factors in Computing Systems (CHI)&lt;/i&gt;, 2024.</t>
+  </si>
+  <si>
+    <t>ohshiro2025audioengineering.pdf</t>
+  </si>
+  <si>
+    <t>Podcasting has evolved as a significant medium where independent creators engage in various production stages, including audio engineering. However, research is limited on how deaf and hard of hearing (dHH) people create podcasts. To address this gap, we conducted interviews with four self-taught dHH podcasters engaged in audio engineering. Our findings reveal how they navigate hearing-related challenges through visual editing techniques, self-taught skill development, and reliance on peer support, while advocating for accessibility. For future directions, we discuss differences between podcast and music audio engineering and recommend integrating AI-powered tools and developing accessible learning resources and environments to support dHH creators.</t>
   </si>
 </sst>
 </file>
@@ -1658,9 +1685,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1698,7 +1725,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1804,7 +1831,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1946,7 +1973,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1954,12 +1981,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R48"/>
+  <dimension ref="A1:R50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" style="2"/>
+    <col min="1" max="1" width="20" style="2" customWidth="1"/>
     <col min="2" max="2" width="17.83203125" customWidth="1"/>
-    <col min="3" max="4" width="76.6640625" customWidth="1"/>
+    <col min="3" max="3" width="76.6640625" customWidth="1"/>
+    <col min="4" max="4" width="27.33203125" customWidth="1"/>
     <col min="6" max="6" width="51.1640625" customWidth="1"/>
     <col min="7" max="7" width="73.33203125" customWidth="1"/>
   </cols>
@@ -3612,6 +3640,61 @@
       </c>
       <c r="R48" t="s">
         <v>289</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A49" s="2">
+        <v>45423</v>
+      </c>
+      <c r="B49" t="s">
+        <v>356</v>
+      </c>
+      <c r="C49" t="s">
+        <v>326</v>
+      </c>
+      <c r="D49" t="s">
+        <v>300</v>
+      </c>
+      <c r="E49" t="s">
+        <v>362</v>
+      </c>
+      <c r="F49" t="s">
+        <v>357</v>
+      </c>
+      <c r="G49" t="s">
+        <v>358</v>
+      </c>
+      <c r="R49" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A50" s="2">
+        <v>45773</v>
+      </c>
+      <c r="B50" t="s">
+        <v>360</v>
+      </c>
+      <c r="C50" t="s">
+        <v>326</v>
+      </c>
+      <c r="D50" t="s">
+        <v>300</v>
+      </c>
+      <c r="E50" t="s">
+        <v>361</v>
+      </c>
+      <c r="F50" t="s">
+        <v>363</v>
+      </c>
+      <c r="G50" t="s">
+        <v>364</v>
+      </c>
+      <c r="L50" t="s">
+        <v>359</v>
+      </c>
+      <c r="R50" t="s">
+        <v>292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added CHI 2026 paper and news item
</commit_message>
<xml_diff>
--- a/markdown_generator/publications.xlsx
+++ b/markdown_generator/publications.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markcartwight/git/sinc-laboratory.github.io/markdown_generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E08266B5-1714-2B4B-BCF8-6CBD08A9AE2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C3C36AB-49C6-4846-BE94-E3E95FF69E87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-2220" yWindow="4300" windowWidth="36000" windowHeight="18220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-1640" yWindow="2000" windowWidth="36000" windowHeight="18220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="publications" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="532" uniqueCount="420">
   <si>
     <t>title</t>
   </si>
@@ -1241,6 +1241,45 @@
   </si>
   <si>
     <t>Frontiers in Computer Science</t>
+  </si>
+  <si>
+    <t>Audiocards: Structured Metadata Improves Audio Language Models for Sound Design</t>
+  </si>
+  <si>
+    <t>sridhar2026audiocards.pdf</t>
+  </si>
+  <si>
+    <t>Sound designers search for sounds in large sound effects libraries using aspects such as sound class or visual context. However, the metadata needed for such search is often missing or incomplete, and requires significant manual effort to add. Existing solutions to automate this task by generating metadata, i.e. captioning, and search using learned embeddings, i.e. text-audio retrieval, are not trained on metadata with the structure and information pertinent to sound design. To this end we propose audiocards, structured metadata grounded in acoustic attributes and sonic descriptors, by exploiting the world knowledge of LLMs. We show that training on audiocards improves downstream text-audio retrieval, descriptive captioning, and metadata generation on professional sound effects libraries. Moreover, audiocards also improve performance on general audio captioning and retrieval over the baseline single-sentence captioning approach. We release a curated dataset of sound effects audiocards to invite further research in audio language modeling for sound design.</t>
+  </si>
+  <si>
+    <t>sridhar2026audiocards_presentation.pdf</t>
+  </si>
+  <si>
+    <t>https://doi.org/10.5281/zenodo.17237181</t>
+  </si>
+  <si>
+    <t>ASFx Eval Audiocards</t>
+  </si>
+  <si>
+    <t>eml,hcap</t>
+  </si>
+  <si>
+    <t>audiocards_overview.png</t>
+  </si>
+  <si>
+    <t>Sridhar, S., Seetharaman, P., Nieto, O., Cartwright, M., Salamon, J. Audiocards: Structured Metadata Improves Audio Language Models for Sound Design. In &lt;i&gt;Proceedings of the IEEE International Conference on Acoustics, Speech and Signal Processing (ICASSP)&lt;/i&gt;, 2026.</t>
+  </si>
+  <si>
+    <t>Like, Comment &amp; Caption: A Decade of Social Media Video Caption Research (2015–2025)</t>
+  </si>
+  <si>
+    <t>Nguyen, H., McDonnell, E., May, L., Druzenko, A., Saifullah, Z., Cartwright, M., Lee, S. Like, Comment &amp; Caption: A Decade of Social Media Video Caption Research (2015–2025). In &lt;i&gt;Proceedings of the ACM Conference on Human Factors in Computing Systems (CHI)&lt;/i&gt;, 2026.</t>
+  </si>
+  <si>
+    <t>nguygen2026like.pdf</t>
+  </si>
+  <si>
+    <t>As video has become the dominant mode of content on platforms such as YouTube, TikTok, and Instagram, captioning has emerged as a critical factor for accessibility, engagement, and visibility. While prior studies have examined different types of social media video captions or communities’ captioning usage, a systematic synthesis has not been undertaken, leading to the risk of proposing interventions that overlook core platform constraints or miss critical accessibility needs. This paper reviews 36 peer-reviewed papers published between 2015 and 2025 across fields such as Human-Computer Interaction (HCI), accessibility, media studies, education, and language learning. We note that captions operate as collective infrastructure co-produced by viewers, creators, and platforms. Deaf and Hard of Hearing (DHH), neurodivergent, and multilingual viewers depend on captions and increasingly expect mechanisms for feedback, while creators face inadequate tool support. Building on these insights, we propose the framework of Participatory Captioning and suggest design implications, highlighting future directions for social media video caption research.</t>
   </si>
 </sst>
 </file>
@@ -1743,7 +1782,7 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="42"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1751,9 +1790,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2110,7 +2146,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R57"/>
+  <dimension ref="A1:R59"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.33203125" style="2" customWidth="1"/>
@@ -4000,10 +4036,10 @@
       <c r="E56" t="s">
         <v>396</v>
       </c>
-      <c r="F56" s="6" t="s">
+      <c r="F56" t="s">
         <v>397</v>
       </c>
-      <c r="G56" s="5" t="s">
+      <c r="G56" t="s">
         <v>398</v>
       </c>
       <c r="R56" t="s">
@@ -4026,14 +4062,81 @@
       <c r="E57" t="s">
         <v>402</v>
       </c>
-      <c r="F57" s="6" t="s">
+      <c r="F57" t="s">
         <v>403</v>
       </c>
-      <c r="G57" s="7" t="s">
+      <c r="G57" t="s">
         <v>404</v>
       </c>
       <c r="R57" t="s">
         <v>405</v>
+      </c>
+    </row>
+    <row r="58" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A58" s="2">
+        <v>46146</v>
+      </c>
+      <c r="B58" t="s">
+        <v>407</v>
+      </c>
+      <c r="C58" t="s">
+        <v>324</v>
+      </c>
+      <c r="D58" t="s">
+        <v>298</v>
+      </c>
+      <c r="E58" t="s">
+        <v>415</v>
+      </c>
+      <c r="F58" t="s">
+        <v>408</v>
+      </c>
+      <c r="G58" t="s">
+        <v>409</v>
+      </c>
+      <c r="H58" t="s">
+        <v>414</v>
+      </c>
+      <c r="J58">
+        <v>100</v>
+      </c>
+      <c r="M58" t="s">
+        <v>410</v>
+      </c>
+      <c r="P58" s="1" t="s">
+        <v>411</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>412</v>
+      </c>
+      <c r="R58" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="59" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A59" s="2">
+        <v>46125</v>
+      </c>
+      <c r="B59" t="s">
+        <v>416</v>
+      </c>
+      <c r="C59" t="s">
+        <v>326</v>
+      </c>
+      <c r="D59" t="s">
+        <v>300</v>
+      </c>
+      <c r="E59" t="s">
+        <v>417</v>
+      </c>
+      <c r="F59" t="s">
+        <v>418</v>
+      </c>
+      <c r="G59" t="s">
+        <v>419</v>
+      </c>
+      <c r="R59" t="s">
+        <v>388</v>
       </c>
     </row>
   </sheetData>
@@ -4046,6 +4149,7 @@
     <hyperlink ref="N20" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
     <hyperlink ref="P22" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
     <hyperlink ref="P33" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="P58" r:id="rId9" xr:uid="{F42196A9-24D4-EF40-9E2D-293465B78BD2}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Fixed naming error in nguyen2026like
</commit_message>
<xml_diff>
--- a/markdown_generator/publications.xlsx
+++ b/markdown_generator/publications.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/markcartwight/git/sinc-laboratory.github.io/markdown_generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C3C36AB-49C6-4846-BE94-E3E95FF69E87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6566C999-7DD6-E741-B414-F3CF0B9B3498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1640" yWindow="2000" windowWidth="36000" windowHeight="18220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5000" yWindow="1560" windowWidth="36000" windowHeight="18220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="publications" sheetId="1" r:id="rId1"/>
@@ -1276,10 +1276,10 @@
     <t>Nguyen, H., McDonnell, E., May, L., Druzenko, A., Saifullah, Z., Cartwright, M., Lee, S. Like, Comment &amp; Caption: A Decade of Social Media Video Caption Research (2015–2025). In &lt;i&gt;Proceedings of the ACM Conference on Human Factors in Computing Systems (CHI)&lt;/i&gt;, 2026.</t>
   </si>
   <si>
-    <t>nguygen2026like.pdf</t>
-  </si>
-  <si>
     <t>As video has become the dominant mode of content on platforms such as YouTube, TikTok, and Instagram, captioning has emerged as a critical factor for accessibility, engagement, and visibility. While prior studies have examined different types of social media video captions or communities’ captioning usage, a systematic synthesis has not been undertaken, leading to the risk of proposing interventions that overlook core platform constraints or miss critical accessibility needs. This paper reviews 36 peer-reviewed papers published between 2015 and 2025 across fields such as Human-Computer Interaction (HCI), accessibility, media studies, education, and language learning. We note that captions operate as collective infrastructure co-produced by viewers, creators, and platforms. Deaf and Hard of Hearing (DHH), neurodivergent, and multilingual viewers depend on captions and increasingly expect mechanisms for feedback, while creators face inadequate tool support. Building on these insights, we propose the framework of Participatory Captioning and suggest design implications, highlighting future directions for social media video caption research.</t>
+  </si>
+  <si>
+    <t>nguyen2026like.pdf</t>
   </si>
 </sst>
 </file>
@@ -4130,10 +4130,10 @@
         <v>417</v>
       </c>
       <c r="F59" t="s">
+        <v>419</v>
+      </c>
+      <c r="G59" t="s">
         <v>418</v>
-      </c>
-      <c r="G59" t="s">
-        <v>419</v>
       </c>
       <c r="R59" t="s">
         <v>388</v>

</xml_diff>